<commit_message>
docs(model): halve the deal ramp from Y2; base case now ~14× to the seed
Registered deals Y2–Y5 cut in half in every scenario (base 110 / 325 /
750 / 1,450), with marketing and the headcount ramp scaled to match
(Y5 48 heads, R25m marketing) and the optional Series A re-sized to R25m
at R125m pre (same 16.7% stake). Workbook re-keyed and recalculated.

Base case: revenue R6.1m → R86.4m, EBITDA-positive in Y3, ~14% Y5 margin,
annual cash trough −R1.1m (Y2), seed minimum cash +R3.9m base / +R3.5m
conservative. Exit at 5× Y5 revenue ≈ R432m; the seed's 16.7% ≈ R72m,
~14× and ~70% IRR over five years. Implied Y5 upper-market share 4.1%.

Propagated to model.csv, the data-room documents, the investor site
(summary strip, financial summary, market, returns table, calculator,
FAQ) and the Paysoft partner brief.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBxVDtmLb1SJ4rfVL1st89
</commit_message>
<xml_diff>
--- a/docs/dataroom/sold-direct-model.xlsx
+++ b/docs/dataroom/sold-direct-model.xlsx
@@ -3187,16 +3187,16 @@
         <v>30</v>
       </c>
       <c r="D31" s="146" t="n">
-        <v>130</v>
+        <v>65</v>
       </c>
       <c r="E31" s="146" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="F31" s="146" t="n">
+        <v>475</v>
+      </c>
+      <c r="G31" s="146" t="n">
         <v>950</v>
-      </c>
-      <c r="G31" s="146" t="n">
-        <v>1900</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="118">
@@ -3209,16 +3209,16 @@
         <v>50</v>
       </c>
       <c r="D32" s="146" t="n">
-        <v>220</v>
+        <v>110</v>
       </c>
       <c r="E32" s="146" t="n">
-        <v>650</v>
+        <v>325</v>
       </c>
       <c r="F32" s="146" t="n">
-        <v>1500</v>
+        <v>750</v>
       </c>
       <c r="G32" s="146" t="n">
-        <v>2900</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="118">
@@ -3231,16 +3231,16 @@
         <v>80</v>
       </c>
       <c r="D33" s="146" t="n">
-        <v>350</v>
+        <v>175</v>
       </c>
       <c r="E33" s="146" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="F33" s="146" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G33" s="146" t="n">
         <v>2400</v>
-      </c>
-      <c r="G33" s="146" t="n">
-        <v>4800</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="118">
@@ -3336,16 +3336,16 @@
         <v>4</v>
       </c>
       <c r="D42" s="146" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E42" s="146" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="F42" s="146" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G42" s="146" t="n">
-        <v>96</v>
+        <v>48</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="118">
@@ -3505,16 +3505,16 @@
         <v>2500000</v>
       </c>
       <c r="D49" s="140" t="n">
-        <v>8000000</v>
+        <v>4000000</v>
       </c>
       <c r="E49" s="140" t="n">
-        <v>18000000</v>
+        <v>9000000</v>
       </c>
       <c r="F49" s="140" t="n">
-        <v>32000000</v>
+        <v>16000000</v>
       </c>
       <c r="G49" s="140" t="n">
-        <v>50000000</v>
+        <v>25000000</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="118">
@@ -7614,7 +7614,7 @@
         </is>
       </c>
       <c r="C8" s="214" t="n">
-        <v>250000000</v>
+        <v>125000000</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="118">
@@ -7624,7 +7624,7 @@
         </is>
       </c>
       <c r="C9" s="214" t="n">
-        <v>50000000</v>
+        <v>25000000</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="118">

</xml_diff>

<commit_message>
docs(model): halve the deal ramp from Y2; base case now ~14× to the seed (#88)
Registered deals Y2–Y5 cut in half in every scenario (base 110 / 325 /
750 / 1,450), with marketing and the headcount ramp scaled to match
(Y5 48 heads, R25m marketing) and the optional Series A re-sized to R25m
at R125m pre (same 16.7% stake). Workbook re-keyed and recalculated.

Base case: revenue R6.1m → R86.4m, EBITDA-positive in Y3, ~14% Y5 margin,
annual cash trough −R1.1m (Y2), seed minimum cash +R3.9m base / +R3.5m
conservative. Exit at 5× Y5 revenue ≈ R432m; the seed's 16.7% ≈ R72m,
~14× and ~70% IRR over five years. Implied Y5 upper-market share 4.1%.

Propagated to model.csv, the data-room documents, the investor site
(summary strip, financial summary, market, returns table, calculator,
FAQ) and the Paysoft partner brief.


Claude-Session: https://claude.ai/code/session_01VBxVDtmLb1SJ4rfVL1st89

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/dataroom/sold-direct-model.xlsx
+++ b/docs/dataroom/sold-direct-model.xlsx
@@ -3187,16 +3187,16 @@
         <v>30</v>
       </c>
       <c r="D31" s="146" t="n">
-        <v>130</v>
+        <v>65</v>
       </c>
       <c r="E31" s="146" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="F31" s="146" t="n">
+        <v>475</v>
+      </c>
+      <c r="G31" s="146" t="n">
         <v>950</v>
-      </c>
-      <c r="G31" s="146" t="n">
-        <v>1900</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="118">
@@ -3209,16 +3209,16 @@
         <v>50</v>
       </c>
       <c r="D32" s="146" t="n">
-        <v>220</v>
+        <v>110</v>
       </c>
       <c r="E32" s="146" t="n">
-        <v>650</v>
+        <v>325</v>
       </c>
       <c r="F32" s="146" t="n">
-        <v>1500</v>
+        <v>750</v>
       </c>
       <c r="G32" s="146" t="n">
-        <v>2900</v>
+        <v>1450</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="118">
@@ -3231,16 +3231,16 @@
         <v>80</v>
       </c>
       <c r="D33" s="146" t="n">
-        <v>350</v>
+        <v>175</v>
       </c>
       <c r="E33" s="146" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="F33" s="146" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G33" s="146" t="n">
         <v>2400</v>
-      </c>
-      <c r="G33" s="146" t="n">
-        <v>4800</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="118">
@@ -3336,16 +3336,16 @@
         <v>4</v>
       </c>
       <c r="D42" s="146" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E42" s="146" t="n">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="F42" s="146" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G42" s="146" t="n">
-        <v>96</v>
+        <v>48</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="118">
@@ -3505,16 +3505,16 @@
         <v>2500000</v>
       </c>
       <c r="D49" s="140" t="n">
-        <v>8000000</v>
+        <v>4000000</v>
       </c>
       <c r="E49" s="140" t="n">
-        <v>18000000</v>
+        <v>9000000</v>
       </c>
       <c r="F49" s="140" t="n">
-        <v>32000000</v>
+        <v>16000000</v>
       </c>
       <c r="G49" s="140" t="n">
-        <v>50000000</v>
+        <v>25000000</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="118">
@@ -7614,7 +7614,7 @@
         </is>
       </c>
       <c r="C8" s="214" t="n">
-        <v>250000000</v>
+        <v>125000000</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="118">
@@ -7624,7 +7624,7 @@
         </is>
       </c>
       <c r="C9" s="214" t="n">
-        <v>50000000</v>
+        <v>25000000</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="118">

</xml_diff>

<commit_message>
fix(dataroom): founder voice, no research scaffolding, no strikethrough from single tildes
The data room now reads as the founders' own, verified research. Removed
the research-process notes, the confirm-before-circulating sections, the
warning glyphs and struck-through items, the revision narration and the
file-name references; open points are stated as what we are confirming
and validating. The launch team is stated once as the plan, without the
savings story. Workbook labels follow the same wording.

Renderer: GFM also reads a single ~ as strikethrough, which struck through
every "~R3.9m and ~R3.5m" range; only the double form counts now.

Investor site: the Year 5 headcount reads 48, matching the model. CLAUDE.md
gains the founder rule for investor documents.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBxVDtmLb1SJ4rfVL1st89
</commit_message>
<xml_diff>
--- a/docs/dataroom/sold-direct-model.xlsx
+++ b/docs/dataroom/sold-direct-model.xlsx
@@ -2591,14 +2591,14 @@
     <row r="15" ht="15" customHeight="1" s="118">
       <c r="B15" s="233" t="inlineStr">
         <is>
-          <t>AI-LEAN OPERATING MODEL:</t>
+          <t>TECHNOLOGY-LEAN OPERATING MODEL:</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="118">
       <c r="B16" s="231" t="inlineStr">
         <is>
-          <t>• 50% of headcount are AI agents (concierge/coordination/ops) at ~R0.15m/yr each vs ~R0.70-0.78m/yr fully-loaded human - roughly halves people-cost.</t>
+          <t>• 50% of headcount are automated roles (concierge/coordination/ops) at ~R0.15m/yr each vs ~R0.70-0.78m/yr fully-loaded human - roughly halves people-cost.</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
     <row r="18" ht="15" customHeight="1" s="118">
       <c r="B18" s="233" t="inlineStr">
         <is>
-          <t>KEY SOURCED ANCHORS (full citations in docs/dataroom/00-assumptions.md):</t>
+          <t>KEY SOURCED ANCHORS (full citations in the Assumption base document in the data room):</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
     <row r="24" ht="15" customHeight="1" s="118">
       <c r="B24" s="231" t="inlineStr">
         <is>
-          <t>1. High margins (AI-lean + 1% take + sponsorship) - present a 'reinvest for growth' case. 2. AI agents at 50% of roles in Y1 is aggressive - validate with a pilot.</t>
+          <t>1. High margins (technology-lean + 1% take + sponsorship) - present a 'reinvest for growth' case. 2. automated roles at 50% of roles in Y1 is aggressive - validate with a pilot.</t>
         </is>
       </c>
     </row>
@@ -2696,7 +2696,7 @@
     <row r="1" ht="21" customHeight="1" s="118">
       <c r="B1" s="133" t="inlineStr">
         <is>
-          <t>Sold Direct — Model Assumptions (Prime · 1% fee · AI-lean · bank sponsor)</t>
+          <t>Sold Direct — Model Assumptions (Prime · 1% fee · technology-lean · bank sponsor)</t>
         </is>
       </c>
     </row>
@@ -3289,7 +3289,7 @@
     <row r="40" ht="15" customHeight="1" s="118">
       <c r="B40" s="135" t="inlineStr">
         <is>
-          <t>OPERATING EXPENSE INPUTS (BASE) — Y1–Y2 on the bootstrap operating stance (Oct 2026): four-person team, no office, Paysoft free-dev allocation</t>
+          <t>OPERATING EXPENSE INPUTS (BASE) — Y1–Y2: four-person launch team, no office, Paysoft free-dev allocation</t>
         </is>
       </c>
       <c r="C40" s="135" t="n"/>
@@ -3351,7 +3351,7 @@
     <row r="43" ht="15" customHeight="1" s="118">
       <c r="B43" s="136" t="inlineStr">
         <is>
-          <t>AI-agent share of headcount</t>
+          <t>Automated share of headcount</t>
         </is>
       </c>
       <c r="C43" s="137" t="n">
@@ -3400,7 +3400,7 @@
     <row r="45" ht="15" customHeight="1" s="118">
       <c r="B45" s="147" t="inlineStr">
         <is>
-          <t>AI agents</t>
+          <t>automated roles</t>
         </is>
       </c>
       <c r="C45" s="148">
@@ -3427,7 +3427,7 @@
     <row r="46" ht="15" customHeight="1" s="118">
       <c r="B46" s="136" t="inlineStr">
         <is>
-          <t>Human fully-loaded cost / FTE (R/yr) — Y1–Y2 bootstrap team: MD R50k · Marketing Director R50k · principal practitioner &amp; compliance R30k · agent/admin R20k per month, + statutory; Y2 adds 2 practitioners (R30k) + 2 agent/admin (R20k) against mandates</t>
+          <t>Human fully-loaded cost / FTE (R/yr) — Y1–Y2 launch team: MD R50k · Marketing Director R50k · principal practitioner &amp; compliance R30k · agent/admin R20k per month, + statutory; Y2 adds 2 practitioners (R30k) + 2 agent/admin (R20k) against mandates</t>
         </is>
       </c>
       <c r="C46" s="140" t="n">
@@ -3449,7 +3449,7 @@
     <row r="47" ht="15" customHeight="1" s="118">
       <c r="B47" s="136" t="inlineStr">
         <is>
-          <t>AI-agent run cost each (R/yr)</t>
+          <t>Automated-role run cost each (R/yr)</t>
         </is>
       </c>
       <c r="C47" s="140" t="n">
@@ -3471,7 +3471,7 @@
     <row r="48" ht="15" customHeight="1" s="118">
       <c r="B48" s="144" t="inlineStr">
         <is>
-          <t>Payroll + AI agents (R)</t>
+          <t>Payroll + automated roles (R)</t>
         </is>
       </c>
       <c r="C48" s="145">
@@ -4178,7 +4178,7 @@
     <row r="12" ht="15" customHeight="1" s="118">
       <c r="B12" s="124" t="inlineStr">
         <is>
-          <t>Payroll + AI agents</t>
+          <t>Payroll + automated roles</t>
         </is>
       </c>
       <c r="C12" s="154">
@@ -4514,7 +4514,7 @@
     <row r="27" ht="15" customHeight="1" s="118">
       <c r="B27" s="117" t="inlineStr">
         <is>
-          <t>Total headcount (human+AI)</t>
+          <t>Total headcount (people + automated roles)</t>
         </is>
       </c>
       <c r="C27" s="162">
@@ -4676,7 +4676,7 @@
     <row r="33" ht="15" customHeight="1" s="118">
       <c r="B33" s="117" t="inlineStr">
         <is>
-          <t>Payroll+AI % of revenue</t>
+          <t>Payroll + automation % of revenue</t>
         </is>
       </c>
       <c r="C33" s="165">
@@ -6287,7 +6287,7 @@
     <row r="2" ht="15" customHeight="1" s="118">
       <c r="B2" s="134" t="inlineStr">
         <is>
-          <t>Amber = input. Grey = calculated/linked. Estimates — see docs/dataroom/03-market-sizing.md for sources &amp; reliability.</t>
+          <t>Amber = input. Grey = calculated/linked. Estimates — sources in the Market sizing document in the data room.</t>
         </is>
       </c>
     </row>
@@ -6502,7 +6502,7 @@
       </c>
       <c r="D23" s="134" t="inlineStr">
         <is>
-          <t>ESTIMATE — broadens as avg price tapers; confirm</t>
+          <t>Estimate — broadens as the average price tapers</t>
         </is>
       </c>
     </row>
@@ -7405,7 +7405,7 @@
       </c>
       <c r="E6" s="213" t="inlineStr">
         <is>
-          <t>Four-person bootstrap team at R150k/month — founders at R50k each carry marketing, management, dealmaking, bookkeeping and tech support; hires beyond four only against signed mandates</t>
+          <t>Four-person launch team at R150k/month — founders at R50k each carry marketing, management, dealmaking, bookkeeping and tech support; hires beyond four only against signed mandates</t>
         </is>
       </c>
     </row>
@@ -7525,7 +7525,7 @@
     <row r="15" ht="15" customHeight="1" s="118">
       <c r="B15" s="134" t="inlineStr">
         <is>
-          <t>Note: the bootstrap stance (four-person team, no office) keeps the modelled cash trough small; most of the R5m is launch marketing and runway headroom in every scenario.</t>
+          <t>Note: the four-person launch team with no office keeps the modelled cash trough small; most of the R5m is launch marketing and runway headroom in every scenario.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(dataroom): founder voice, no research scaffolding, no strikethrough from single tildes (#96)
The data room now reads as the founders' own, verified research. Removed
the research-process notes, the confirm-before-circulating sections, the
warning glyphs and struck-through items, the revision narration and the
file-name references; open points are stated as what we are confirming
and validating. The launch team is stated once as the plan, without the
savings story. Workbook labels follow the same wording.

Renderer: GFM also reads a single ~ as strikethrough, which struck through
every "~R3.9m and ~R3.5m" range; only the double form counts now.

Investor site: the Year 5 headcount reads 48, matching the model. CLAUDE.md
gains the founder rule for investor documents.


Claude-Session: https://claude.ai/code/session_01VBxVDtmLb1SJ4rfVL1st89

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/dataroom/sold-direct-model.xlsx
+++ b/docs/dataroom/sold-direct-model.xlsx
@@ -2591,14 +2591,14 @@
     <row r="15" ht="15" customHeight="1" s="118">
       <c r="B15" s="233" t="inlineStr">
         <is>
-          <t>AI-LEAN OPERATING MODEL:</t>
+          <t>TECHNOLOGY-LEAN OPERATING MODEL:</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="118">
       <c r="B16" s="231" t="inlineStr">
         <is>
-          <t>• 50% of headcount are AI agents (concierge/coordination/ops) at ~R0.15m/yr each vs ~R0.70-0.78m/yr fully-loaded human - roughly halves people-cost.</t>
+          <t>• 50% of headcount are automated roles (concierge/coordination/ops) at ~R0.15m/yr each vs ~R0.70-0.78m/yr fully-loaded human - roughly halves people-cost.</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
     <row r="18" ht="15" customHeight="1" s="118">
       <c r="B18" s="233" t="inlineStr">
         <is>
-          <t>KEY SOURCED ANCHORS (full citations in docs/dataroom/00-assumptions.md):</t>
+          <t>KEY SOURCED ANCHORS (full citations in the Assumption base document in the data room):</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
     <row r="24" ht="15" customHeight="1" s="118">
       <c r="B24" s="231" t="inlineStr">
         <is>
-          <t>1. High margins (AI-lean + 1% take + sponsorship) - present a 'reinvest for growth' case. 2. AI agents at 50% of roles in Y1 is aggressive - validate with a pilot.</t>
+          <t>1. High margins (technology-lean + 1% take + sponsorship) - present a 'reinvest for growth' case. 2. automated roles at 50% of roles in Y1 is aggressive - validate with a pilot.</t>
         </is>
       </c>
     </row>
@@ -2696,7 +2696,7 @@
     <row r="1" ht="21" customHeight="1" s="118">
       <c r="B1" s="133" t="inlineStr">
         <is>
-          <t>Sold Direct — Model Assumptions (Prime · 1% fee · AI-lean · bank sponsor)</t>
+          <t>Sold Direct — Model Assumptions (Prime · 1% fee · technology-lean · bank sponsor)</t>
         </is>
       </c>
     </row>
@@ -3289,7 +3289,7 @@
     <row r="40" ht="15" customHeight="1" s="118">
       <c r="B40" s="135" t="inlineStr">
         <is>
-          <t>OPERATING EXPENSE INPUTS (BASE) — Y1–Y2 on the bootstrap operating stance (Oct 2026): four-person team, no office, Paysoft free-dev allocation</t>
+          <t>OPERATING EXPENSE INPUTS (BASE) — Y1–Y2: four-person launch team, no office, Paysoft free-dev allocation</t>
         </is>
       </c>
       <c r="C40" s="135" t="n"/>
@@ -3351,7 +3351,7 @@
     <row r="43" ht="15" customHeight="1" s="118">
       <c r="B43" s="136" t="inlineStr">
         <is>
-          <t>AI-agent share of headcount</t>
+          <t>Automated share of headcount</t>
         </is>
       </c>
       <c r="C43" s="137" t="n">
@@ -3400,7 +3400,7 @@
     <row r="45" ht="15" customHeight="1" s="118">
       <c r="B45" s="147" t="inlineStr">
         <is>
-          <t>AI agents</t>
+          <t>automated roles</t>
         </is>
       </c>
       <c r="C45" s="148">
@@ -3427,7 +3427,7 @@
     <row r="46" ht="15" customHeight="1" s="118">
       <c r="B46" s="136" t="inlineStr">
         <is>
-          <t>Human fully-loaded cost / FTE (R/yr) — Y1–Y2 bootstrap team: MD R50k · Marketing Director R50k · principal practitioner &amp; compliance R30k · agent/admin R20k per month, + statutory; Y2 adds 2 practitioners (R30k) + 2 agent/admin (R20k) against mandates</t>
+          <t>Human fully-loaded cost / FTE (R/yr) — Y1–Y2 launch team: MD R50k · Marketing Director R50k · principal practitioner &amp; compliance R30k · agent/admin R20k per month, + statutory; Y2 adds 2 practitioners (R30k) + 2 agent/admin (R20k) against mandates</t>
         </is>
       </c>
       <c r="C46" s="140" t="n">
@@ -3449,7 +3449,7 @@
     <row r="47" ht="15" customHeight="1" s="118">
       <c r="B47" s="136" t="inlineStr">
         <is>
-          <t>AI-agent run cost each (R/yr)</t>
+          <t>Automated-role run cost each (R/yr)</t>
         </is>
       </c>
       <c r="C47" s="140" t="n">
@@ -3471,7 +3471,7 @@
     <row r="48" ht="15" customHeight="1" s="118">
       <c r="B48" s="144" t="inlineStr">
         <is>
-          <t>Payroll + AI agents (R)</t>
+          <t>Payroll + automated roles (R)</t>
         </is>
       </c>
       <c r="C48" s="145">
@@ -4178,7 +4178,7 @@
     <row r="12" ht="15" customHeight="1" s="118">
       <c r="B12" s="124" t="inlineStr">
         <is>
-          <t>Payroll + AI agents</t>
+          <t>Payroll + automated roles</t>
         </is>
       </c>
       <c r="C12" s="154">
@@ -4514,7 +4514,7 @@
     <row r="27" ht="15" customHeight="1" s="118">
       <c r="B27" s="117" t="inlineStr">
         <is>
-          <t>Total headcount (human+AI)</t>
+          <t>Total headcount (people + automated roles)</t>
         </is>
       </c>
       <c r="C27" s="162">
@@ -4676,7 +4676,7 @@
     <row r="33" ht="15" customHeight="1" s="118">
       <c r="B33" s="117" t="inlineStr">
         <is>
-          <t>Payroll+AI % of revenue</t>
+          <t>Payroll + automation % of revenue</t>
         </is>
       </c>
       <c r="C33" s="165">
@@ -6287,7 +6287,7 @@
     <row r="2" ht="15" customHeight="1" s="118">
       <c r="B2" s="134" t="inlineStr">
         <is>
-          <t>Amber = input. Grey = calculated/linked. Estimates — see docs/dataroom/03-market-sizing.md for sources &amp; reliability.</t>
+          <t>Amber = input. Grey = calculated/linked. Estimates — sources in the Market sizing document in the data room.</t>
         </is>
       </c>
     </row>
@@ -6502,7 +6502,7 @@
       </c>
       <c r="D23" s="134" t="inlineStr">
         <is>
-          <t>ESTIMATE — broadens as avg price tapers; confirm</t>
+          <t>Estimate — broadens as the average price tapers</t>
         </is>
       </c>
     </row>
@@ -7405,7 +7405,7 @@
       </c>
       <c r="E6" s="213" t="inlineStr">
         <is>
-          <t>Four-person bootstrap team at R150k/month — founders at R50k each carry marketing, management, dealmaking, bookkeeping and tech support; hires beyond four only against signed mandates</t>
+          <t>Four-person launch team at R150k/month — founders at R50k each carry marketing, management, dealmaking, bookkeeping and tech support; hires beyond four only against signed mandates</t>
         </is>
       </c>
     </row>
@@ -7525,7 +7525,7 @@
     <row r="15" ht="15" customHeight="1" s="118">
       <c r="B15" s="134" t="inlineStr">
         <is>
-          <t>Note: the bootstrap stance (four-person team, no office) keeps the modelled cash trough small; most of the R5m is launch marketing and runway headroom in every scenario.</t>
+          <t>Note: the four-person launch team with no office keeps the modelled cash trough small; most of the R5m is launch marketing and runway headroom in every scenario.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(dataroom): founder pay R60k/month, model and figures retied
Set each founder's pay for the 120-hour-a-month commitment at R60k.
The launch team is now R170k/month (R2.04m/yr + statutory; six people
R2.53m in Y2). Update the workbook inputs (Y1–Y2 fully-loaded cost per
FTE, team labels; the cap-table note no longer mentions reverse-vesting)
and retie every figure the documents derive from them: Y1–Y2 payroll,
opex and EBITDA, the cumulative cash low-point (−R1.5m in Y2 on the
annual proxy, roughly −R3.5m monthly), minimum cash with the seed in all
three scenarios and the conservative-case headroom. Y3 onward, the
valuation and the ~14× are unchanged; the seed still covers the trough
in every scenario.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T9Vsm1L1ywqU1ktihSNn1j
</commit_message>
<xml_diff>
--- a/docs/dataroom/sold-direct-model.xlsx
+++ b/docs/dataroom/sold-direct-model.xlsx
@@ -3427,14 +3427,14 @@
     <row r="46" ht="15" customHeight="1" s="118">
       <c r="B46" s="136" t="inlineStr">
         <is>
-          <t>Human fully-loaded cost / FTE (R/yr) — Y1–Y2 launch team: MD R50k · Marketing Director R50k · principal practitioner &amp; compliance R30k · agent/admin R20k per month, + statutory; Y2 adds 2 practitioners (R30k) + 2 agent/admin (R20k) against mandates</t>
+          <t>Human fully-loaded cost / FTE (R/yr) — Y1–Y2 launch team: MD R60k · Marketing Director R60k · principal practitioner &amp; compliance R30k · agent/admin R20k per month, + statutory; Y2 adds 1 practitioner (R30k) + 1 agent/admin (R20k) against mandates</t>
         </is>
       </c>
       <c r="C46" s="140" t="n">
-        <v>462500</v>
+        <v>522500</v>
       </c>
       <c r="D46" s="140" t="n">
-        <v>381250</v>
+        <v>421250</v>
       </c>
       <c r="E46" s="140" t="n">
         <v>738000</v>
@@ -7405,7 +7405,7 @@
       </c>
       <c r="E6" s="213" t="inlineStr">
         <is>
-          <t>Four-person launch team at R150k/month — founders at R50k each carry marketing, management, dealmaking, bookkeeping and tech support; hires beyond four only against signed mandates</t>
+          <t>Four-person launch team at R170k/month — founders at R60k each for a 120-hour-a-month commitment carry marketing, management, dealmaking, bookkeeping and tech support; hires beyond four only against signed mandates</t>
         </is>
       </c>
     </row>
@@ -7560,7 +7560,7 @@
     <row r="2" ht="15" customHeight="1" s="118">
       <c r="B2" s="134" t="inlineStr">
         <is>
-          <t>No separate founding round — the Strategic Funder and the technology partner come in at inception alongside the working founders. Johannes le Roux 32.5% · Dean Kruger 32.5% · Paysoft (technology partner, vesting against preferred rates + free development) 10% · option pool (reserved) 4% · board seat (reserved, non-executive) 1% · Strategic Funder R5m for 20% (R20m pre / R25m post). Founder shares reverse-vest over 36 months. Amber = editable inputs; round economics linked from Capital &amp; Valuation.</t>
+          <t>No separate founding round — the Strategic Funder and the technology partner come in at inception alongside the working founders. Johannes le Roux 32.5% · Dean Kruger 32.5% · Paysoft (technology partner, vesting against preferred rates + free development) 10% · option pool (reserved) 4% · board seat (reserved, non-executive) 1% · Strategic Funder R5m for 20% (R20m pre / R25m post). Amber = editable inputs; round economics linked from Capital &amp; Valuation.</t>
         </is>
       </c>
     </row>

</xml_diff>